<commit_message>
Checking in Hearts data
</commit_message>
<xml_diff>
--- a/src/test/resources/TestDriver/Hearst/ReferenceData/RefData_Hearst.xlsx
+++ b/src/test/resources/TestDriver/Hearst/ReferenceData/RefData_Hearst.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b68cc7b829e61597/Desktop/Hearst_Project/Sandbox/RefData/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7" documentId="13_ncr:1_{8B35AA18-597C-43D1-99E2-2B2D168188B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0862C481-5C70-4E39-A616-393A6916013A}"/>
+  <xr:revisionPtr revIDLastSave="15" documentId="13_ncr:1_{8B35AA18-597C-43D1-99E2-2B2D168188B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B90DF04B-0383-4CDC-A2CC-ED758CA35D51}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Transactions" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="71">
   <si>
     <t>Name</t>
   </si>
@@ -248,6 +248,12 @@
   </si>
   <si>
     <t>Total_Revenue</t>
+  </si>
+  <si>
+    <t>Allocated_Revenue</t>
+  </si>
+  <si>
+    <t>New_Booking</t>
   </si>
 </sst>
 </file>
@@ -531,7 +537,7 @@
   <sheetPr>
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="45.28515625" customWidth="1"/>
@@ -595,6 +601,20 @@
       </c>
       <c r="D4" s="3">
         <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="B5" s="3">
+        <v>0</v>
+      </c>
+      <c r="C5" s="3">
+        <v>1</v>
+      </c>
+      <c r="D5" s="3">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -930,7 +950,7 @@
   <sheetPr>
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="67.7109375" style="1" customWidth="1"/>
@@ -1009,6 +1029,14 @@
       </c>
       <c r="B9" s="1" t="s">
         <v>68</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>70</v>
       </c>
     </row>
   </sheetData>

</xml_diff>